<commit_message>
Added Permissions and Improved Contract logic
</commit_message>
<xml_diff>
--- a/ContratosYReembolsos/Data/SeedData/Branches.xlsx
+++ b/ContratosYReembolsos/Data/SeedData/Branches.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\desarrollo\Documents\SeedData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4FC6C9EC-1015-4DC0-AC3D-6A7F34C7E770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7173EF3-658B-4442-B403-75005CC521C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{FA51A0F0-52BA-4549-AE29-9B3C6DA60EB1}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="310">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="488" uniqueCount="309">
   <si>
     <t>Id</t>
   </si>
@@ -61,9 +61,6 @@
   </si>
   <si>
     <t>Email</t>
-  </si>
-  <si>
-    <t>HasWakeService</t>
   </si>
   <si>
     <t>064 - 5261</t>
@@ -973,8 +970,16 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -1014,7 +1019,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
@@ -1023,14 +1028,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="3">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
+  <dxfs count="2">
     <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
@@ -1063,18 +1066,17 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4E628CC1-85D8-438E-AB2E-9C07971F14AB}" name="Tabla11" displayName="Tabla11" ref="A1:I81" totalsRowShown="0">
-  <autoFilter ref="A1:I81" xr:uid="{E56CAAAA-E9D9-4A29-B93F-5332B48EAC07}"/>
-  <tableColumns count="9">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{4E628CC1-85D8-438E-AB2E-9C07971F14AB}" name="Tabla11" displayName="Tabla11" ref="A1:H81" totalsRowShown="0">
+  <autoFilter ref="A1:H81" xr:uid="{E56CAAAA-E9D9-4A29-B93F-5332B48EAC07}"/>
+  <tableColumns count="8">
     <tableColumn id="1" xr3:uid="{B727090F-CC28-4C39-95BD-9E7A171F4819}" name="Id"/>
     <tableColumn id="2" xr3:uid="{C56E108B-B33F-469A-9766-CB3D5382463E}" name="Name"/>
-    <tableColumn id="3" xr3:uid="{38714165-B749-44CE-9F2E-08A4B18D26F1}" name="UbigeoId" dataDxfId="2"/>
+    <tableColumn id="3" xr3:uid="{38714165-B749-44CE-9F2E-08A4B18D26F1}" name="UbigeoId" dataDxfId="1"/>
     <tableColumn id="4" xr3:uid="{777EB4BC-F8A7-4D16-B44E-3F14B9A6BEDB}" name="Code"/>
     <tableColumn id="5" xr3:uid="{5546D51E-4A21-4E77-85B2-F68A79EF5A95}" name="Address"/>
     <tableColumn id="6" xr3:uid="{2D5F42F7-EC67-4DAF-BD37-D9634B72507E}" name="Phone"/>
     <tableColumn id="7" xr3:uid="{99C49CF0-BA07-4EF6-8048-B668605BB2D7}" name="Email"/>
-    <tableColumn id="8" xr3:uid="{424CA1D4-AF75-42FC-9A67-12C036F9DEB9}" name="IsActive" dataDxfId="1"/>
-    <tableColumn id="9" xr3:uid="{D9CD682D-AF0E-4056-A710-072496EA69D4}" name="HasWakeService" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{424CA1D4-AF75-42FC-9A67-12C036F9DEB9}" name="IsActive" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1377,18 +1379,18 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0E2EABC-64CB-4DD0-822A-34CFF8C119C8}">
-  <dimension ref="A1:I81"/>
+  <dimension ref="A1:H81"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="47" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="11.42578125" style="1" customWidth="1"/>
     <col min="4" max="4" width="24.28515625" customWidth="1"/>
-    <col min="5" max="7" width="11.42578125" customWidth="1"/>
+    <col min="5" max="5" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="6" max="7" width="11.42578125" customWidth="1"/>
     <col min="8" max="8" width="10.28515625" style="7" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="18" style="7" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1413,2328 +1415,2085 @@
       <c r="H1" s="7" t="s">
         <v>2</v>
       </c>
-      <c r="I1" s="7" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D2" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="E2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="F2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H2" s="7">
         <v>1</v>
       </c>
-      <c r="I2" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E3" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H3" s="7">
         <v>1</v>
       </c>
-      <c r="I3" s="7">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H4" s="7">
         <v>1</v>
       </c>
-      <c r="I4" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5">
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="D5" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E5" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="F5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="G5" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H5" s="7">
         <v>1</v>
       </c>
-      <c r="I5" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6">
         <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D6" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="G6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H6" s="7">
         <v>1</v>
       </c>
-      <c r="I6" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7">
         <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="D7" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="E7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="G7" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H7" s="7">
         <v>1</v>
       </c>
-      <c r="I7" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8">
         <v>7</v>
       </c>
       <c r="B8" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D8" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F8" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="G8" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H8" s="7">
         <v>1</v>
       </c>
-      <c r="I8" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
+        <v>146</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>273</v>
+      </c>
+      <c r="D9" s="8" t="s">
+        <v>70</v>
+      </c>
+      <c r="E9" t="s">
+        <v>144</v>
+      </c>
+      <c r="F9" t="s">
         <v>147</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>274</v>
-      </c>
-      <c r="D9" t="s">
-        <v>71</v>
-      </c>
-      <c r="E9" t="s">
-        <v>145</v>
-      </c>
-      <c r="F9" t="s">
-        <v>148</v>
-      </c>
       <c r="G9" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H9" s="7">
         <v>1</v>
       </c>
-      <c r="I9" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10">
         <v>9</v>
       </c>
       <c r="B10" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
       <c r="D10" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G10" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H10" s="7">
         <v>1</v>
       </c>
-      <c r="I10" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
       <c r="D11" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G11" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H11" s="7">
         <v>1</v>
       </c>
-      <c r="I11" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12">
         <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="D12" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G12" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H12" s="7">
         <v>1</v>
       </c>
-      <c r="I12" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13">
         <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
       <c r="D13" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F13" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="G13" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H13" s="7">
         <v>1</v>
       </c>
-      <c r="I13" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14">
         <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="D14" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F14" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="G14" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H14" s="7">
         <v>1</v>
       </c>
-      <c r="I14" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15">
         <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
       <c r="D15" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="E15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F15" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="G15" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H15" s="7">
         <v>1</v>
       </c>
-      <c r="I15" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16">
         <v>15</v>
       </c>
       <c r="B16" t="s">
+        <v>156</v>
+      </c>
+      <c r="C16" s="2" t="s">
         <v>157</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>158</v>
-      </c>
       <c r="D16" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="E16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F16" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G16" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H16" s="7">
         <v>1</v>
       </c>
-      <c r="I16" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17">
         <v>16</v>
       </c>
       <c r="B17" t="s">
+        <v>158</v>
+      </c>
+      <c r="C17" s="2" t="s">
         <v>159</v>
       </c>
-      <c r="C17" s="2" t="s">
+      <c r="D17" t="s">
+        <v>78</v>
+      </c>
+      <c r="E17" t="s">
         <v>160</v>
       </c>
-      <c r="D17" t="s">
-        <v>79</v>
-      </c>
-      <c r="E17" t="s">
-        <v>161</v>
-      </c>
       <c r="F17" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="G17" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H17" s="7">
         <v>1</v>
       </c>
-      <c r="I17" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18">
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
       <c r="D18" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="G18" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H18" s="7">
         <v>1</v>
       </c>
-      <c r="I18" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19">
         <v>18</v>
       </c>
       <c r="B19" t="s">
+        <v>162</v>
+      </c>
+      <c r="C19" s="2" t="s">
         <v>163</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>164</v>
-      </c>
       <c r="D19" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F19" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="G19" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H19" s="7">
         <v>1</v>
       </c>
-      <c r="I19" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20">
         <v>19</v>
       </c>
       <c r="B20" t="s">
+        <v>164</v>
+      </c>
+      <c r="C20" s="1" t="s">
         <v>165</v>
       </c>
-      <c r="C20" s="1" t="s">
-        <v>166</v>
-      </c>
       <c r="D20" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="E20" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F20" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="G20" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H20" s="7">
         <v>1</v>
       </c>
-      <c r="I20" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21">
         <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
       <c r="D21" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="E21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F21" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G21" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H21" s="7">
         <v>1</v>
       </c>
-      <c r="I21" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22">
         <v>21</v>
       </c>
       <c r="B22" t="s">
+        <v>167</v>
+      </c>
+      <c r="C22" s="1" t="s">
         <v>168</v>
       </c>
-      <c r="C22" s="1" t="s">
-        <v>169</v>
-      </c>
       <c r="D22" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="E22" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F22" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G22" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H22" s="7">
         <v>1</v>
       </c>
-      <c r="I22" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23">
         <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="C23" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="D23" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F23" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="G23" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H23" s="7">
         <v>1</v>
       </c>
-      <c r="I23" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24">
         <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="D24" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="E24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G24" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H24" s="7">
         <v>1</v>
       </c>
-      <c r="I24" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25">
         <v>24</v>
       </c>
       <c r="B25" t="s">
+        <v>171</v>
+      </c>
+      <c r="C25" s="2" t="s">
         <v>172</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>173</v>
-      </c>
       <c r="D25" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="G25" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H25" s="7">
         <v>1</v>
       </c>
-      <c r="I25" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26">
         <v>25</v>
       </c>
       <c r="B26" t="s">
+        <v>173</v>
+      </c>
+      <c r="C26" s="2" t="s">
         <v>174</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>175</v>
-      </c>
       <c r="D26" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="E26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G26" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H26" s="7">
         <v>1</v>
       </c>
-      <c r="I26" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27">
         <v>26</v>
       </c>
       <c r="B27" s="3" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="C27" s="2" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
       <c r="D27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="E27" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F27" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="G27" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H27" s="7">
         <v>1</v>
       </c>
-      <c r="I27" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A28">
         <v>27</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="C28" s="2" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="D28" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F28" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="G28" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H28" s="7">
         <v>1</v>
       </c>
-      <c r="I28" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A29">
         <v>28</v>
       </c>
       <c r="B29" s="3" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="C29" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
       <c r="D29" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E29" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F29" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="G29" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H29" s="7">
         <v>1</v>
       </c>
-      <c r="I29" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A30">
         <v>29</v>
       </c>
       <c r="B30" s="3" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
       <c r="D30" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F30" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="G30" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H30" s="7">
         <v>1</v>
       </c>
-      <c r="I30" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A31">
         <v>30</v>
       </c>
       <c r="B31" s="3" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="C31" s="2" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
       <c r="D31" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="E31" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F31" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="G31" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H31" s="7">
         <v>1</v>
       </c>
-      <c r="I31" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A32">
         <v>31</v>
       </c>
       <c r="B32" s="3" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="C32" s="2" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
       <c r="D32" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="E32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F32" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="G32" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H32" s="7">
         <v>1</v>
       </c>
-      <c r="I32" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="33" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A33">
         <v>32</v>
       </c>
       <c r="B33" t="s">
+        <v>181</v>
+      </c>
+      <c r="C33" s="1" t="s">
         <v>182</v>
       </c>
-      <c r="C33" s="1" t="s">
-        <v>183</v>
-      </c>
       <c r="D33" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="E33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F33" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G33" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H33" s="7">
         <v>1</v>
       </c>
-      <c r="I33" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="34" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A34">
         <v>33</v>
       </c>
       <c r="B34" t="s">
+        <v>183</v>
+      </c>
+      <c r="C34" s="1" t="s">
         <v>184</v>
       </c>
-      <c r="C34" s="1" t="s">
+      <c r="D34" t="s">
+        <v>95</v>
+      </c>
+      <c r="E34" t="s">
         <v>185</v>
       </c>
-      <c r="D34" t="s">
-        <v>96</v>
-      </c>
-      <c r="E34" t="s">
-        <v>186</v>
-      </c>
       <c r="F34" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G34" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H34" s="7">
         <v>1</v>
       </c>
-      <c r="I34" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="35" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A35">
         <v>34</v>
       </c>
       <c r="B35" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
       <c r="D35" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="E35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F35" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="G35" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H35" s="7">
         <v>1</v>
       </c>
-      <c r="I35" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="36" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A36">
         <v>35</v>
       </c>
       <c r="B36" s="3" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="D36" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G36" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H36" s="7">
         <v>1</v>
       </c>
-      <c r="I36" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="37" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A37">
         <v>36</v>
       </c>
       <c r="B37" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="D37" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="E37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G37" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H37" s="7">
         <v>1</v>
       </c>
-      <c r="I37" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="38" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A38">
         <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="D38" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="E38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F38" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="G38" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H38" s="7">
         <v>1</v>
       </c>
-      <c r="I38" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="39" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A39">
         <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="D39" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="E39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F39" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G39" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H39" s="7">
         <v>1</v>
       </c>
-      <c r="I39" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40">
         <v>39</v>
       </c>
       <c r="B40" t="s">
+        <v>193</v>
+      </c>
+      <c r="C40" s="2" t="s">
         <v>194</v>
       </c>
-      <c r="C40" s="2" t="s">
+      <c r="D40" t="s">
+        <v>101</v>
+      </c>
+      <c r="E40" t="s">
         <v>195</v>
       </c>
-      <c r="D40" t="s">
-        <v>102</v>
-      </c>
-      <c r="E40" t="s">
-        <v>196</v>
-      </c>
       <c r="F40" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="G40" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H40" s="7">
         <v>1</v>
       </c>
-      <c r="I40" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="41" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A41">
         <v>40</v>
       </c>
       <c r="B41" s="3" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="D41" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="E41" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F41" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G41" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H41" s="7">
         <v>1</v>
       </c>
-      <c r="I41" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A42">
         <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="C42" s="2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D42" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="E42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F42" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="G42" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H42" s="7">
         <v>1</v>
       </c>
-      <c r="I42" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="43" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A43">
         <v>42</v>
       </c>
       <c r="B43" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D43" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="E43" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="F43" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G43" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H43" s="7">
         <v>1</v>
       </c>
-      <c r="I43" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="44" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A44">
         <v>43</v>
       </c>
       <c r="B44" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="C44" s="2" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="D44" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="E44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F44" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G44" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H44" s="7">
         <v>1</v>
       </c>
-      <c r="I44" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="45" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A45">
         <v>44</v>
       </c>
       <c r="B45" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>292</v>
+        <v>291</v>
       </c>
       <c r="D45" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E45" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F45" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="G45" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H45" s="7">
         <v>1</v>
       </c>
-      <c r="I45" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="46" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A46">
         <v>45</v>
       </c>
       <c r="B46" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="C46" s="2" t="s">
-        <v>293</v>
+        <v>292</v>
       </c>
       <c r="D46" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G46" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H46" s="7">
         <v>1</v>
       </c>
-      <c r="I46" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="47" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A47">
         <v>46</v>
       </c>
       <c r="B47" s="3" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="C47" s="2" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="D47" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="E47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G47" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H47" s="7">
         <v>1</v>
       </c>
-      <c r="I47" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="48" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A48">
         <v>47</v>
       </c>
       <c r="B48" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="C48" s="2" t="s">
-        <v>295</v>
+        <v>294</v>
       </c>
       <c r="D48" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="E48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F48" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="G48" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H48" s="7">
         <v>1</v>
       </c>
-      <c r="I48" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="49" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A49">
         <v>48</v>
       </c>
       <c r="B49" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>296</v>
+        <v>295</v>
       </c>
       <c r="D49" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E49" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F49" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="G49" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H49" s="7">
         <v>1</v>
       </c>
-      <c r="I49" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="50" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A50">
         <v>49</v>
       </c>
       <c r="B50" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="C50" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
       <c r="D50" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E50" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F50" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G50" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H50" s="7">
         <v>1</v>
       </c>
-      <c r="I50" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="51" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A51">
         <v>50</v>
       </c>
       <c r="B51" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D51" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F51" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="G51" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H51" s="7">
         <v>1</v>
       </c>
-      <c r="I51" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="52" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A52">
         <v>51</v>
       </c>
       <c r="B52" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C52" s="2" t="s">
-        <v>298</v>
+        <v>297</v>
       </c>
       <c r="D52" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E52" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F52" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G52" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H52" s="7">
         <v>1</v>
       </c>
-      <c r="I52" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="53" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A53">
         <v>52</v>
       </c>
       <c r="B53" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C53" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="D53" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E53" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F53" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G53" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H53" s="7">
         <v>1</v>
       </c>
-      <c r="I53" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="54" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A54">
         <v>53</v>
       </c>
       <c r="B54" t="s">
+        <v>212</v>
+      </c>
+      <c r="C54" s="2" t="s">
         <v>213</v>
       </c>
-      <c r="C54" s="2" t="s">
-        <v>214</v>
-      </c>
       <c r="D54" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="E54" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F54" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G54" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H54" s="7">
         <v>1</v>
       </c>
-      <c r="I54" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="55" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A55">
         <v>54</v>
       </c>
       <c r="B55" t="s">
+        <v>221</v>
+      </c>
+      <c r="C55" s="1" t="s">
         <v>222</v>
       </c>
-      <c r="C55" s="1" t="s">
-        <v>223</v>
-      </c>
       <c r="D55" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="E55" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F55" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="G55" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H55" s="7">
         <v>1</v>
       </c>
-      <c r="I55" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A56">
         <v>55</v>
       </c>
       <c r="B56" s="3" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="C56" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="D56" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G56" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H56" s="7">
         <v>1</v>
       </c>
-      <c r="I56" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A57">
         <v>56</v>
       </c>
       <c r="B57" t="s">
+        <v>224</v>
+      </c>
+      <c r="C57" s="2" t="s">
         <v>225</v>
       </c>
-      <c r="C57" s="2" t="s">
+      <c r="D57" t="s">
+        <v>121</v>
+      </c>
+      <c r="E57" t="s">
         <v>226</v>
       </c>
-      <c r="D57" t="s">
-        <v>122</v>
-      </c>
-      <c r="E57" t="s">
-        <v>227</v>
-      </c>
       <c r="F57" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G57" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H57" s="7">
         <v>1</v>
       </c>
-      <c r="I57" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A58">
         <v>57</v>
       </c>
       <c r="B58" t="s">
+        <v>227</v>
+      </c>
+      <c r="C58" s="2" t="s">
         <v>228</v>
       </c>
-      <c r="C58" s="2" t="s">
-        <v>229</v>
-      </c>
       <c r="D58" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E58" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F58" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G58" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H58" s="7">
         <v>1</v>
       </c>
-      <c r="I58" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A59">
         <v>58</v>
       </c>
       <c r="B59" t="s">
+        <v>229</v>
+      </c>
+      <c r="C59" s="2" t="s">
         <v>230</v>
       </c>
-      <c r="C59" s="2" t="s">
-        <v>231</v>
-      </c>
       <c r="D59" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E59" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F59" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G59" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H59" s="7">
         <v>1</v>
       </c>
-      <c r="I59" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A60">
         <v>59</v>
       </c>
       <c r="B60" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="C60" s="2" t="s">
-        <v>299</v>
+        <v>298</v>
       </c>
       <c r="D60" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E60" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F60" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="G60" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H60" s="7">
         <v>1</v>
       </c>
-      <c r="I60" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A61">
         <v>60</v>
       </c>
       <c r="B61" t="s">
+        <v>232</v>
+      </c>
+      <c r="C61" s="2" t="s">
         <v>233</v>
       </c>
-      <c r="C61" s="2" t="s">
-        <v>234</v>
-      </c>
       <c r="D61" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E61" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F61" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G61" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H61" s="7">
         <v>1</v>
       </c>
-      <c r="I61" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A62">
         <v>61</v>
       </c>
       <c r="B62" t="s">
+        <v>234</v>
+      </c>
+      <c r="C62" s="1" t="s">
         <v>235</v>
       </c>
-      <c r="C62" s="1" t="s">
-        <v>236</v>
-      </c>
       <c r="D62" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G62" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H62" s="7">
         <v>1</v>
       </c>
-      <c r="I62" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A63">
         <v>62</v>
       </c>
       <c r="B63" t="s">
+        <v>236</v>
+      </c>
+      <c r="C63" s="2" t="s">
         <v>237</v>
       </c>
-      <c r="C63" s="2" t="s">
+      <c r="D63" t="s">
+        <v>127</v>
+      </c>
+      <c r="E63" t="s">
+        <v>144</v>
+      </c>
+      <c r="F63" t="s">
         <v>238</v>
       </c>
-      <c r="D63" t="s">
-        <v>128</v>
-      </c>
-      <c r="E63" t="s">
-        <v>145</v>
-      </c>
-      <c r="F63" t="s">
-        <v>239</v>
-      </c>
       <c r="G63" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H63" s="7">
         <v>1</v>
       </c>
-      <c r="I63" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A64">
         <v>63</v>
       </c>
       <c r="B64" t="s">
+        <v>239</v>
+      </c>
+      <c r="C64" s="2" t="s">
         <v>240</v>
       </c>
-      <c r="C64" s="2" t="s">
-        <v>241</v>
-      </c>
       <c r="D64" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E64" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F64" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G64" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H64" s="7">
         <v>1</v>
       </c>
-      <c r="I64" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A65">
         <v>64</v>
       </c>
       <c r="B65" t="s">
+        <v>241</v>
+      </c>
+      <c r="C65" s="2" t="s">
         <v>242</v>
       </c>
-      <c r="C65" s="2" t="s">
-        <v>243</v>
-      </c>
       <c r="D65" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="E65" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F65" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="G65" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H65" s="7">
         <v>1</v>
       </c>
-      <c r="I65" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A66">
         <v>65</v>
       </c>
       <c r="B66" t="s">
+        <v>243</v>
+      </c>
+      <c r="C66" s="2" t="s">
         <v>244</v>
       </c>
-      <c r="C66" s="2" t="s">
-        <v>245</v>
-      </c>
       <c r="D66" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G66" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H66" s="7">
         <v>1</v>
       </c>
-      <c r="I66" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="67" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A67">
         <v>66</v>
       </c>
       <c r="B67" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>300</v>
+        <v>299</v>
       </c>
       <c r="D67" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G67" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H67" s="7">
         <v>1</v>
       </c>
-      <c r="I67" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A68">
         <v>67</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="C68" s="2" t="s">
-        <v>301</v>
+        <v>300</v>
       </c>
       <c r="D68" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E68" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F68" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="G68" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H68" s="7">
         <v>1</v>
       </c>
-      <c r="I68" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A69">
         <v>68</v>
       </c>
       <c r="B69" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="C69" s="2" t="s">
-        <v>302</v>
+        <v>301</v>
       </c>
       <c r="D69" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E69" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F69" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="G69" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H69" s="7">
         <v>1</v>
       </c>
-      <c r="I69" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A70">
         <v>69</v>
       </c>
       <c r="B70" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C70" s="2" t="s">
-        <v>303</v>
+        <v>302</v>
       </c>
       <c r="D70" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E70" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F70" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G70" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H70" s="7">
         <v>1</v>
       </c>
-      <c r="I70" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A71">
         <v>70</v>
       </c>
       <c r="B71" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>261</v>
+        <v>260</v>
       </c>
       <c r="D71" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="E71" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F71" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="G71" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H71" s="7">
         <v>1</v>
       </c>
-      <c r="I71" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A72">
         <v>71</v>
       </c>
       <c r="B72" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>256</v>
+        <v>255</v>
       </c>
       <c r="D72" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E72" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F72" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="G72" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H72" s="7">
         <v>1</v>
       </c>
-      <c r="I72" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A73">
         <v>72</v>
       </c>
       <c r="B73" t="s">
-        <v>254</v>
+        <v>253</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>252</v>
+        <v>251</v>
       </c>
       <c r="D73" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E73" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F73" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G73" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H73" s="7">
         <v>1</v>
       </c>
-      <c r="I73" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A74">
         <v>73</v>
       </c>
       <c r="B74" t="s">
-        <v>255</v>
+        <v>254</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="D74" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E74" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F74" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G74" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H74" s="7">
         <v>1</v>
       </c>
-      <c r="I74" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A75">
         <v>74</v>
       </c>
       <c r="B75" s="4" t="s">
+        <v>256</v>
+      </c>
+      <c r="C75" s="1" t="s">
         <v>257</v>
       </c>
-      <c r="C75" s="1" t="s">
-        <v>258</v>
-      </c>
       <c r="D75" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E75" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F75" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G75" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H75" s="7">
         <v>1</v>
       </c>
-      <c r="I75" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A76">
         <v>75</v>
       </c>
       <c r="B76" s="4" t="s">
-        <v>259</v>
+        <v>258</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>258</v>
+        <v>257</v>
       </c>
       <c r="D76" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E76" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F76" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G76" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H76" s="7">
         <v>1</v>
       </c>
-      <c r="I76" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A77">
         <v>76</v>
       </c>
       <c r="B77" t="s">
-        <v>260</v>
+        <v>259</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="D77" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E77" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F77" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="G77" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H77" s="7">
         <v>1</v>
       </c>
-      <c r="I77" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A78">
         <v>77</v>
       </c>
       <c r="B78" t="s">
+        <v>261</v>
+      </c>
+      <c r="C78" s="1" t="s">
         <v>262</v>
       </c>
-      <c r="C78" s="1" t="s">
-        <v>263</v>
-      </c>
       <c r="D78" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E78" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F78" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G78" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H78" s="7">
         <v>1</v>
       </c>
-      <c r="I78" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="79" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A79">
         <v>78</v>
       </c>
       <c r="B79" t="s">
+        <v>263</v>
+      </c>
+      <c r="C79" s="2" t="s">
         <v>264</v>
       </c>
-      <c r="C79" s="2" t="s">
+      <c r="D79" t="s">
+        <v>141</v>
+      </c>
+      <c r="E79" t="s">
         <v>265</v>
       </c>
-      <c r="D79" t="s">
-        <v>142</v>
-      </c>
-      <c r="E79" t="s">
-        <v>266</v>
-      </c>
       <c r="F79" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G79" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H79" s="7">
         <v>1</v>
       </c>
-      <c r="I79" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="80" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A80">
         <v>79</v>
       </c>
       <c r="B80" t="s">
+        <v>266</v>
+      </c>
+      <c r="C80" s="2" t="s">
         <v>267</v>
       </c>
-      <c r="C80" s="2" t="s">
-        <v>268</v>
-      </c>
       <c r="D80" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="E80" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F80" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="G80" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H80" s="7">
         <v>1</v>
       </c>
-      <c r="I80" s="7">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.25">
+    </row>
+    <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81">
         <v>80</v>
       </c>
       <c r="B81" s="3" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="C81" s="2" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="D81" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="E81" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="F81" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="G81" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="H81" s="7">
         <v>1</v>
-      </c>
-      <c r="I81" s="7">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>